<commit_message>
Empate: WYB172896960 -> WYB173790694
</commit_message>
<xml_diff>
--- a/overrides.xlsx
+++ b/overrides.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -595,6 +595,43 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>REVERTIDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WYB172896960</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>WYB173790694</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-05-28 06:35:34</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Falló 1ra y 2da visita</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>operador</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Enviado: jueves, 14 de mayo de 2026 16:23</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ACTIVA</t>
         </is>
       </c>
     </row>

</xml_diff>